<commit_message>
Expand survey dataset to 110 respondents (adding 28 CSE and 30 AIML students) and regenerate PDF report
</commit_message>
<xml_diff>
--- a/survey_responses (1).xlsx
+++ b/survey_responses (1).xlsx
@@ -398,14 +398,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:N115"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="22.83203125" customWidth="1"/>
     <col min="4" max="4" width="36.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
     <col min="8" max="8" width="18.83203125" customWidth="1"/>
     <col min="9" max="9" width="26.83203125" customWidth="1"/>
@@ -428,7 +428,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Author: Kabir | Target Population: University Students Across Multiple Academic Disciplines</v>
+        <v>Author: Kabir | Target Population: University Students Across Diverse Academic Disciplines</v>
       </c>
     </row>
     <row r="5">
@@ -2763,20 +2763,2572 @@
         <v>None provided</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58">
+        <v>53</v>
+      </c>
+      <c r="B58" t="str">
+        <v>2026-10-08T09:20:15.000Z</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Prachi Singhania</v>
+      </c>
+      <c r="D58" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E58" t="str">
+        <v>9819234812</v>
+      </c>
+      <c r="F58" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G58" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H58">
+        <v>4</v>
+      </c>
+      <c r="I58" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J58">
+        <v>4</v>
+      </c>
+      <c r="K58">
+        <v>4</v>
+      </c>
+      <c r="L58">
+        <v>4</v>
+      </c>
+      <c r="M58" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N58" t="str">
+        <v>helpful for finding syntax errors in C++</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>54</v>
+      </c>
+      <c r="B59" t="str">
+        <v>2026-10-08T10:14:22.000Z</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Prasanna Kollu</v>
+      </c>
+      <c r="D59" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E59" t="str">
+        <v>9849012845</v>
+      </c>
+      <c r="F59" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H59">
+        <v>3</v>
+      </c>
+      <c r="I59" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J59">
+        <v>4</v>
+      </c>
+      <c r="K59">
+        <v>4</v>
+      </c>
+      <c r="L59">
+        <v>4</v>
+      </c>
+      <c r="M59" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N59" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>55</v>
+      </c>
+      <c r="B60" t="str">
+        <v>2026-10-08T11:05:40.000Z</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Purva Derkar</v>
+      </c>
+      <c r="D60" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E60" t="str">
+        <v>9765412903</v>
+      </c>
+      <c r="F60" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H60">
+        <v>4</v>
+      </c>
+      <c r="I60" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J60">
+        <v>4</v>
+      </c>
+      <c r="K60">
+        <v>3</v>
+      </c>
+      <c r="L60">
+        <v>4</v>
+      </c>
+      <c r="M60" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N60" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>56</v>
+      </c>
+      <c r="B61" t="str">
+        <v>2026-10-08T11:45:10.000Z</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Rama Sudeshna</v>
+      </c>
+      <c r="D61" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E61" t="str">
+        <v>9823109482</v>
+      </c>
+      <c r="F61" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H61">
+        <v>4</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J61">
+        <v>5</v>
+      </c>
+      <c r="K61">
+        <v>4</v>
+      </c>
+      <c r="L61">
+        <v>5</v>
+      </c>
+      <c r="M61" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N61" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>57</v>
+      </c>
+      <c r="B62" t="str">
+        <v>2026-10-08T12:30:05.000Z</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Rathneshvaran I</v>
+      </c>
+      <c r="D62" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E62" t="str">
+        <v>9940128471</v>
+      </c>
+      <c r="F62" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G62" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H62">
+        <v>3</v>
+      </c>
+      <c r="I62" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J62">
+        <v>4</v>
+      </c>
+      <c r="K62">
+        <v>4</v>
+      </c>
+      <c r="L62">
+        <v>4</v>
+      </c>
+      <c r="M62" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N62" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>58</v>
+      </c>
+      <c r="B63" t="str">
+        <v>2026-10-08T14:15:30.000Z</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Remalle Sathvik Theophilus</v>
+      </c>
+      <c r="D63" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E63" t="str">
+        <v>9848019284</v>
+      </c>
+      <c r="F63" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G63" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H63">
+        <v>4</v>
+      </c>
+      <c r="I63" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J63">
+        <v>4</v>
+      </c>
+      <c r="K63">
+        <v>4</v>
+      </c>
+      <c r="L63">
+        <v>4</v>
+      </c>
+      <c r="M63" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N63" t="str">
+        <v>mostly use it for lab assignments</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>59</v>
+      </c>
+      <c r="B64" t="str">
+        <v>2026-10-08T15:02:18.000Z</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Riddhi Agarwal</v>
+      </c>
+      <c r="D64" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E64" t="str">
+        <v>9711048291</v>
+      </c>
+      <c r="F64" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G64" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H64">
+        <v>4</v>
+      </c>
+      <c r="I64" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J64">
+        <v>3</v>
+      </c>
+      <c r="K64">
+        <v>4</v>
+      </c>
+      <c r="L64">
+        <v>3</v>
+      </c>
+      <c r="M64" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N64" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>60</v>
+      </c>
+      <c r="B65" t="str">
+        <v>2026-10-08T16:20:45.000Z</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Rudra Kumar</v>
+      </c>
+      <c r="D65" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E65" t="str">
+        <v>9810482910</v>
+      </c>
+      <c r="F65" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G65" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H65">
+        <v>3</v>
+      </c>
+      <c r="I65" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J65">
+        <v>4</v>
+      </c>
+      <c r="K65">
+        <v>4</v>
+      </c>
+      <c r="L65">
+        <v>4</v>
+      </c>
+      <c r="M65" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N65" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>61</v>
+      </c>
+      <c r="B66" t="str">
+        <v>2026-10-09T09:10:12.000Z</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Saathvik Mahalsa Koppolu</v>
+      </c>
+      <c r="D66" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E66" t="str">
+        <v>9989018472</v>
+      </c>
+      <c r="F66" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H66">
+        <v>4</v>
+      </c>
+      <c r="I66" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J66">
+        <v>4</v>
+      </c>
+      <c r="K66">
+        <v>4</v>
+      </c>
+      <c r="L66">
+        <v>4</v>
+      </c>
+      <c r="M66" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N66" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>62</v>
+      </c>
+      <c r="B67" t="str">
+        <v>2026-10-09T10:05:33.000Z</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Sahasra Devunuri</v>
+      </c>
+      <c r="D67" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E67" t="str">
+        <v>9866019284</v>
+      </c>
+      <c r="F67" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G67" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H67">
+        <v>4</v>
+      </c>
+      <c r="I67" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J67">
+        <v>4</v>
+      </c>
+      <c r="K67">
+        <v>3</v>
+      </c>
+      <c r="L67">
+        <v>4</v>
+      </c>
+      <c r="M67" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N67" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>63</v>
+      </c>
+      <c r="B68" t="str">
+        <v>2026-10-09T11:22:19.000Z</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Samarth Samanekar</v>
+      </c>
+      <c r="D68" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E68" t="str">
+        <v>9741029384</v>
+      </c>
+      <c r="F68" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G68" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H68">
+        <v>4</v>
+      </c>
+      <c r="I68" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J68">
+        <v>5</v>
+      </c>
+      <c r="K68">
+        <v>4</v>
+      </c>
+      <c r="L68">
+        <v>5</v>
+      </c>
+      <c r="M68" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N68" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>64</v>
+      </c>
+      <c r="B69" t="str">
+        <v>2026-10-09T12:40:02.000Z</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Sambhaji Sandip Dungahu</v>
+      </c>
+      <c r="D69" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E69" t="str">
+        <v>9822019482</v>
+      </c>
+      <c r="F69" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G69" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H69">
+        <v>3</v>
+      </c>
+      <c r="I69" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J69">
+        <v>4</v>
+      </c>
+      <c r="K69">
+        <v>4</v>
+      </c>
+      <c r="L69">
+        <v>4</v>
+      </c>
+      <c r="M69" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N69" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>65</v>
+      </c>
+      <c r="B70" t="str">
+        <v>2026-10-09T14:15:20.000Z</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Sanjay K</v>
+      </c>
+      <c r="D70" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E70" t="str">
+        <v>9900128471</v>
+      </c>
+      <c r="F70" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H70">
+        <v>4</v>
+      </c>
+      <c r="I70" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J70">
+        <v>3</v>
+      </c>
+      <c r="K70">
+        <v>4</v>
+      </c>
+      <c r="L70">
+        <v>3</v>
+      </c>
+      <c r="M70" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N70" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>66</v>
+      </c>
+      <c r="B71" t="str">
+        <v>2026-10-09T15:30:11.000Z</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Sharanya Mishra</v>
+      </c>
+      <c r="D71" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E71" t="str">
+        <v>9818049281</v>
+      </c>
+      <c r="F71" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G71" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H71">
+        <v>4</v>
+      </c>
+      <c r="I71" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J71">
+        <v>4</v>
+      </c>
+      <c r="K71">
+        <v>4</v>
+      </c>
+      <c r="L71">
+        <v>4</v>
+      </c>
+      <c r="M71" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N71" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>67</v>
+      </c>
+      <c r="B72" t="str">
+        <v>2026-10-09T16:45:50.000Z</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Shardul Yadav</v>
+      </c>
+      <c r="D72" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E72" t="str">
+        <v>9873019284</v>
+      </c>
+      <c r="F72" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G72" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H72">
+        <v>4</v>
+      </c>
+      <c r="I72" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J72">
+        <v>4</v>
+      </c>
+      <c r="K72">
+        <v>4</v>
+      </c>
+      <c r="L72">
+        <v>4</v>
+      </c>
+      <c r="M72" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N72" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>68</v>
+      </c>
+      <c r="B73" t="str">
+        <v>2026-10-10T09:18:24.000Z</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Shaurya Mittal</v>
+      </c>
+      <c r="D73" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E73" t="str">
+        <v>9811029482</v>
+      </c>
+      <c r="F73" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G73" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H73">
+        <v>4</v>
+      </c>
+      <c r="I73" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J73">
+        <v>4</v>
+      </c>
+      <c r="K73">
+        <v>4</v>
+      </c>
+      <c r="L73">
+        <v>4</v>
+      </c>
+      <c r="M73" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N73" t="str">
+        <v>good for regex and bash commands</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>69</v>
+      </c>
+      <c r="B74" t="str">
+        <v>2026-10-10T10:40:12.000Z</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Shivam Singh</v>
+      </c>
+      <c r="D74" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E74" t="str">
+        <v>9792018472</v>
+      </c>
+      <c r="F74" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G74" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H74">
+        <v>3</v>
+      </c>
+      <c r="I74" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J74">
+        <v>4</v>
+      </c>
+      <c r="K74">
+        <v>4</v>
+      </c>
+      <c r="L74">
+        <v>4</v>
+      </c>
+      <c r="M74" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N74" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>70</v>
+      </c>
+      <c r="B75" t="str">
+        <v>2026-10-10T11:55:03.000Z</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Shreyash Singh</v>
+      </c>
+      <c r="D75" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E75" t="str">
+        <v>9839018274</v>
+      </c>
+      <c r="F75" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H75">
+        <v>4</v>
+      </c>
+      <c r="I75" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J75">
+        <v>4</v>
+      </c>
+      <c r="K75">
+        <v>4</v>
+      </c>
+      <c r="L75">
+        <v>4</v>
+      </c>
+      <c r="M75" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N75" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>71</v>
+      </c>
+      <c r="B76" t="str">
+        <v>2026-10-10T13:10:44.000Z</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Sidharth Sood</v>
+      </c>
+      <c r="D76" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E76" t="str">
+        <v>9816029384</v>
+      </c>
+      <c r="F76" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G76" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H76">
+        <v>4</v>
+      </c>
+      <c r="I76" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J76">
+        <v>5</v>
+      </c>
+      <c r="K76">
+        <v>4</v>
+      </c>
+      <c r="L76">
+        <v>5</v>
+      </c>
+      <c r="M76" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N76" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>72</v>
+      </c>
+      <c r="B77" t="str">
+        <v>2026-10-10T14:25:30.000Z</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Ananey Sharma</v>
+      </c>
+      <c r="D77" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E77" t="str">
+        <v>9872019482</v>
+      </c>
+      <c r="F77" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G77" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H77">
+        <v>4</v>
+      </c>
+      <c r="I77" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J77">
+        <v>4</v>
+      </c>
+      <c r="K77">
+        <v>3</v>
+      </c>
+      <c r="L77">
+        <v>4</v>
+      </c>
+      <c r="M77" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N77" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>73</v>
+      </c>
+      <c r="B78" t="str">
+        <v>2026-10-10T15:50:18.000Z</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Lakshay Sethia</v>
+      </c>
+      <c r="D78" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E78" t="str">
+        <v>9829018472</v>
+      </c>
+      <c r="F78" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G78" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H78">
+        <v>4</v>
+      </c>
+      <c r="I78" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J78">
+        <v>4</v>
+      </c>
+      <c r="K78">
+        <v>5</v>
+      </c>
+      <c r="L78">
+        <v>4</v>
+      </c>
+      <c r="M78" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N78" t="str">
+        <v>saves time on boilerplate react code</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>74</v>
+      </c>
+      <c r="B79" t="str">
+        <v>2026-10-11T09:30:15.000Z</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Kadire Venkata Susankar Reddy</v>
+      </c>
+      <c r="D79" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E79" t="str">
+        <v>9949018274</v>
+      </c>
+      <c r="F79" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G79" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H79">
+        <v>3</v>
+      </c>
+      <c r="I79" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J79">
+        <v>4</v>
+      </c>
+      <c r="K79">
+        <v>4</v>
+      </c>
+      <c r="L79">
+        <v>4</v>
+      </c>
+      <c r="M79" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N79" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>75</v>
+      </c>
+      <c r="B80" t="str">
+        <v>2026-10-11T10:45:22.000Z</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Nihanth Reddy Pannala</v>
+      </c>
+      <c r="D80" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E80" t="str">
+        <v>9848129482</v>
+      </c>
+      <c r="F80" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G80" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H80">
+        <v>4</v>
+      </c>
+      <c r="I80" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J80">
+        <v>4</v>
+      </c>
+      <c r="K80">
+        <v>4</v>
+      </c>
+      <c r="L80">
+        <v>4</v>
+      </c>
+      <c r="M80" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N80" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>76</v>
+      </c>
+      <c r="B81" t="str">
+        <v>2026-10-11T12:10:04.000Z</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Rao Vanshika Prashant</v>
+      </c>
+      <c r="D81" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E81" t="str">
+        <v>9820492810</v>
+      </c>
+      <c r="F81" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G81" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H81">
+        <v>4</v>
+      </c>
+      <c r="I81" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J81">
+        <v>3</v>
+      </c>
+      <c r="K81">
+        <v>4</v>
+      </c>
+      <c r="L81">
+        <v>3</v>
+      </c>
+      <c r="M81" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N81" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>77</v>
+      </c>
+      <c r="B82" t="str">
+        <v>2026-10-11T13:35:48.000Z</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Harshit Yadav</v>
+      </c>
+      <c r="D82" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E82" t="str">
+        <v>9871029482</v>
+      </c>
+      <c r="F82" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G82" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H82">
+        <v>4</v>
+      </c>
+      <c r="I82" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J82">
+        <v>4</v>
+      </c>
+      <c r="K82">
+        <v>4</v>
+      </c>
+      <c r="L82">
+        <v>4</v>
+      </c>
+      <c r="M82" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N82" t="str">
+        <v>good when stuck on dsa problems</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <v>78</v>
+      </c>
+      <c r="B83" t="str">
+        <v>2026-10-11T15:00:20.000Z</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Shivam Mishra</v>
+      </c>
+      <c r="D83" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E83" t="str">
+        <v>9838019482</v>
+      </c>
+      <c r="F83" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G83" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H83">
+        <v>3</v>
+      </c>
+      <c r="I83" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J83">
+        <v>4</v>
+      </c>
+      <c r="K83">
+        <v>4</v>
+      </c>
+      <c r="L83">
+        <v>4</v>
+      </c>
+      <c r="M83" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N83" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>79</v>
+      </c>
+      <c r="B84" t="str">
+        <v>2026-10-11T16:15:40.000Z</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Sudati Nikhil Rao</v>
+      </c>
+      <c r="D84" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E84" t="str">
+        <v>9963018274</v>
+      </c>
+      <c r="F84" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G84" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H84">
+        <v>4</v>
+      </c>
+      <c r="I84" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J84">
+        <v>4</v>
+      </c>
+      <c r="K84">
+        <v>4</v>
+      </c>
+      <c r="L84">
+        <v>4</v>
+      </c>
+      <c r="M84" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N84" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>80</v>
+      </c>
+      <c r="B85" t="str">
+        <v>2026-10-11T17:30:10.000Z</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Vuyyuru Abhirami</v>
+      </c>
+      <c r="D85" t="str">
+        <v>B.Tech Computer Science &amp; Engineering</v>
+      </c>
+      <c r="E85" t="str">
+        <v>9849201948</v>
+      </c>
+      <c r="F85" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G85" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H85">
+        <v>4</v>
+      </c>
+      <c r="I85" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J85">
+        <v>4</v>
+      </c>
+      <c r="K85">
+        <v>4</v>
+      </c>
+      <c r="L85">
+        <v>4</v>
+      </c>
+      <c r="M85" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N85" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86">
+        <v>81</v>
+      </c>
+      <c r="B86" t="str">
+        <v>2026-10-12T09:05:14.000Z</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Mantena Gagan Sri Varma</v>
+      </c>
+      <c r="D86" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E86" t="str">
+        <v>9989128472</v>
+      </c>
+      <c r="F86" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G86" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H86">
+        <v>4</v>
+      </c>
+      <c r="I86" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J86">
+        <v>4</v>
+      </c>
+      <c r="K86">
+        <v>4</v>
+      </c>
+      <c r="L86">
+        <v>4</v>
+      </c>
+      <c r="M86" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N86" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>82</v>
+      </c>
+      <c r="B87" t="str">
+        <v>2026-10-12T10:18:22.000Z</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Manthena Naga Sri Rohan</v>
+      </c>
+      <c r="D87" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E87" t="str">
+        <v>9848239104</v>
+      </c>
+      <c r="F87" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G87" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H87">
+        <v>3</v>
+      </c>
+      <c r="I87" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J87">
+        <v>4</v>
+      </c>
+      <c r="K87">
+        <v>4</v>
+      </c>
+      <c r="L87">
+        <v>4</v>
+      </c>
+      <c r="M87" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N87" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>83</v>
+      </c>
+      <c r="B88" t="str">
+        <v>2026-10-12T11:30:05.000Z</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Martala Harsha Vardhan Reddy</v>
+      </c>
+      <c r="D88" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E88" t="str">
+        <v>9949382019</v>
+      </c>
+      <c r="F88" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G88" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H88">
+        <v>4</v>
+      </c>
+      <c r="I88" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J88">
+        <v>5</v>
+      </c>
+      <c r="K88">
+        <v>4</v>
+      </c>
+      <c r="L88">
+        <v>5</v>
+      </c>
+      <c r="M88" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N88" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>84</v>
+      </c>
+      <c r="B89" t="str">
+        <v>2026-10-12T12:45:10.000Z</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Masula Megha Chayana</v>
+      </c>
+      <c r="D89" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E89" t="str">
+        <v>9866102948</v>
+      </c>
+      <c r="F89" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G89" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H89">
+        <v>4</v>
+      </c>
+      <c r="I89" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J89">
+        <v>4</v>
+      </c>
+      <c r="K89">
+        <v>4</v>
+      </c>
+      <c r="L89">
+        <v>4</v>
+      </c>
+      <c r="M89" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N89" t="str">
+        <v>helps explain complex math in machine learning</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>85</v>
+      </c>
+      <c r="B90" t="str">
+        <v>2026-10-12T14:02:40.000Z</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Mayank Panigrahi</v>
+      </c>
+      <c r="D90" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E90" t="str">
+        <v>9437019284</v>
+      </c>
+      <c r="F90" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G90" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H90">
+        <v>4</v>
+      </c>
+      <c r="I90" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J90">
+        <v>4</v>
+      </c>
+      <c r="K90">
+        <v>4</v>
+      </c>
+      <c r="L90">
+        <v>4</v>
+      </c>
+      <c r="M90" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N90" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>86</v>
+      </c>
+      <c r="B91" t="str">
+        <v>2026-10-12T15:20:15.000Z</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Maydhaansh Nanda</v>
+      </c>
+      <c r="D91" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E91" t="str">
+        <v>9810129482</v>
+      </c>
+      <c r="F91" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G91" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H91">
+        <v>3</v>
+      </c>
+      <c r="I91" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J91">
+        <v>4</v>
+      </c>
+      <c r="K91">
+        <v>4</v>
+      </c>
+      <c r="L91">
+        <v>4</v>
+      </c>
+      <c r="M91" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N91" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>87</v>
+      </c>
+      <c r="B92" t="str">
+        <v>2026-10-12T16:35:28.000Z</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Md Aali Rahman</v>
+      </c>
+      <c r="D92" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E92" t="str">
+        <v>9835019284</v>
+      </c>
+      <c r="F92" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G92" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H92">
+        <v>4</v>
+      </c>
+      <c r="I92" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J92">
+        <v>4</v>
+      </c>
+      <c r="K92">
+        <v>3</v>
+      </c>
+      <c r="L92">
+        <v>4</v>
+      </c>
+      <c r="M92" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N92" t="str">
+        <v>dont memorize pandas methods now</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>88</v>
+      </c>
+      <c r="B93" t="str">
+        <v>2026-10-12T17:50:44.000Z</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Mihir Kalway</v>
+      </c>
+      <c r="D93" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E93" t="str">
+        <v>9910948271</v>
+      </c>
+      <c r="F93" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G93" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H93">
+        <v>4</v>
+      </c>
+      <c r="I93" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J93">
+        <v>4</v>
+      </c>
+      <c r="K93">
+        <v>4</v>
+      </c>
+      <c r="L93">
+        <v>4</v>
+      </c>
+      <c r="M93" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N93" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
+        <v>89</v>
+      </c>
+      <c r="B94" t="str">
+        <v>2026-10-13T09:12:00.000Z</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Mithi Jaiswal</v>
+      </c>
+      <c r="D94" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E94" t="str">
+        <v>9826019284</v>
+      </c>
+      <c r="F94" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G94" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H94">
+        <v>4</v>
+      </c>
+      <c r="I94" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J94">
+        <v>3</v>
+      </c>
+      <c r="K94">
+        <v>4</v>
+      </c>
+      <c r="L94">
+        <v>3</v>
+      </c>
+      <c r="M94" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N94" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95">
+        <v>90</v>
+      </c>
+      <c r="B95" t="str">
+        <v>2026-10-13T10:25:18.000Z</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Mohammad Saalim</v>
+      </c>
+      <c r="D95" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E95" t="str">
+        <v>9849301928</v>
+      </c>
+      <c r="F95" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G95" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H95">
+        <v>4</v>
+      </c>
+      <c r="I95" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J95">
+        <v>4</v>
+      </c>
+      <c r="K95">
+        <v>4</v>
+      </c>
+      <c r="L95">
+        <v>4</v>
+      </c>
+      <c r="M95" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N95" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <v>91</v>
+      </c>
+      <c r="B96" t="str">
+        <v>2026-10-13T11:40:30.000Z</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Mohammad Zeeshan Bin Sadiq</v>
+      </c>
+      <c r="D96" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E96" t="str">
+        <v>9848392019</v>
+      </c>
+      <c r="F96" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G96" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H96">
+        <v>4</v>
+      </c>
+      <c r="I96" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J96">
+        <v>5</v>
+      </c>
+      <c r="K96">
+        <v>4</v>
+      </c>
+      <c r="L96">
+        <v>5</v>
+      </c>
+      <c r="M96" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N96" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>92</v>
+      </c>
+      <c r="B97" t="str">
+        <v>2026-10-13T12:55:10.000Z</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Mohammed Ali</v>
+      </c>
+      <c r="D97" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E97" t="str">
+        <v>9885019284</v>
+      </c>
+      <c r="F97" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H97">
+        <v>3</v>
+      </c>
+      <c r="I97" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J97">
+        <v>4</v>
+      </c>
+      <c r="K97">
+        <v>4</v>
+      </c>
+      <c r="L97">
+        <v>4</v>
+      </c>
+      <c r="M97" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N97" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>93</v>
+      </c>
+      <c r="B98" t="str">
+        <v>2026-10-13T14:10:45.000Z</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Mohammed Ayman</v>
+      </c>
+      <c r="D98" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E98" t="str">
+        <v>9849401928</v>
+      </c>
+      <c r="F98" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G98" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H98">
+        <v>4</v>
+      </c>
+      <c r="I98" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J98">
+        <v>4</v>
+      </c>
+      <c r="K98">
+        <v>4</v>
+      </c>
+      <c r="L98">
+        <v>4</v>
+      </c>
+      <c r="M98" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N98" t="str">
+        <v>useful for debugging pytorch models</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>94</v>
+      </c>
+      <c r="B99" t="str">
+        <v>2026-10-13T15:24:20.000Z</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Mohammed Zaid</v>
+      </c>
+      <c r="D99" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E99" t="str">
+        <v>9949501928</v>
+      </c>
+      <c r="F99" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G99" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H99">
+        <v>4</v>
+      </c>
+      <c r="I99" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J99">
+        <v>4</v>
+      </c>
+      <c r="K99">
+        <v>3</v>
+      </c>
+      <c r="L99">
+        <v>4</v>
+      </c>
+      <c r="M99" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N99" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>95</v>
+      </c>
+      <c r="B100" t="str">
+        <v>2026-10-13T16:38:05.000Z</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Mohd Tausifur Rahman</v>
+      </c>
+      <c r="D100" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E100" t="str">
+        <v>9835129482</v>
+      </c>
+      <c r="F100" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G100" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H100">
+        <v>3</v>
+      </c>
+      <c r="I100" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J100">
+        <v>4</v>
+      </c>
+      <c r="K100">
+        <v>4</v>
+      </c>
+      <c r="L100">
+        <v>4</v>
+      </c>
+      <c r="M100" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N100" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>96</v>
+      </c>
+      <c r="B101" t="str">
+        <v>2026-10-13T17:45:12.000Z</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Muddasani Riya Reddy</v>
+      </c>
+      <c r="D101" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E101" t="str">
+        <v>9866201948</v>
+      </c>
+      <c r="F101" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G101" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H101">
+        <v>4</v>
+      </c>
+      <c r="I101" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J101">
+        <v>4</v>
+      </c>
+      <c r="K101">
+        <v>4</v>
+      </c>
+      <c r="L101">
+        <v>4</v>
+      </c>
+      <c r="M101" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N101" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>97</v>
+      </c>
+      <c r="B102" t="str">
+        <v>2026-10-14T08:50:30.000Z</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Mugula Sahan Yadav</v>
+      </c>
+      <c r="D102" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E102" t="str">
+        <v>9989201948</v>
+      </c>
+      <c r="F102" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G102" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H102">
+        <v>4</v>
+      </c>
+      <c r="I102" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J102">
+        <v>4</v>
+      </c>
+      <c r="K102">
+        <v>4</v>
+      </c>
+      <c r="L102">
+        <v>4</v>
+      </c>
+      <c r="M102" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N102" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>98</v>
+      </c>
+      <c r="B103" t="str">
+        <v>2026-10-14T09:15:22.000Z</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Mulakala Manoj Sri Sathya Charan</v>
+      </c>
+      <c r="D103" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E103" t="str">
+        <v>9848401928</v>
+      </c>
+      <c r="F103" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G103" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H103">
+        <v>4</v>
+      </c>
+      <c r="I103" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J103">
+        <v>5</v>
+      </c>
+      <c r="K103">
+        <v>5</v>
+      </c>
+      <c r="L103">
+        <v>5</v>
+      </c>
+      <c r="M103" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N103" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>99</v>
+      </c>
+      <c r="B104" t="str">
+        <v>2026-10-14T09:30:10.000Z</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Muthoju Keertan</v>
+      </c>
+      <c r="D104" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E104" t="str">
+        <v>9949601928</v>
+      </c>
+      <c r="F104" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H104">
+        <v>4</v>
+      </c>
+      <c r="I104" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J104">
+        <v>4</v>
+      </c>
+      <c r="K104">
+        <v>4</v>
+      </c>
+      <c r="L104">
+        <v>4</v>
+      </c>
+      <c r="M104" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N104" t="str">
+        <v>makes writing documentation faster</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>100</v>
+      </c>
+      <c r="B105" t="str">
+        <v>2026-10-14T09:42:15.000Z</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Nabiha Fatima</v>
+      </c>
+      <c r="D105" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E105" t="str">
+        <v>9885129482</v>
+      </c>
+      <c r="F105" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G105" t="str">
+        <v>Weekly</v>
+      </c>
+      <c r="H105">
+        <v>4</v>
+      </c>
+      <c r="I105" t="str">
+        <v>Remained the Same</v>
+      </c>
+      <c r="J105">
+        <v>3</v>
+      </c>
+      <c r="K105">
+        <v>4</v>
+      </c>
+      <c r="L105">
+        <v>3</v>
+      </c>
+      <c r="M105" t="str">
+        <v>No change</v>
+      </c>
+      <c r="N105" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>101</v>
+      </c>
+      <c r="B106" t="str">
+        <v>2026-10-14T09:55:40.000Z</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Charith</v>
+      </c>
+      <c r="D106" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E106" t="str">
+        <v>9963102948</v>
+      </c>
+      <c r="F106" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G106" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H106">
+        <v>3</v>
+      </c>
+      <c r="I106" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J106">
+        <v>4</v>
+      </c>
+      <c r="K106">
+        <v>4</v>
+      </c>
+      <c r="L106">
+        <v>4</v>
+      </c>
+      <c r="M106" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N106" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107">
+        <v>102</v>
+      </c>
+      <c r="B107" t="str">
+        <v>2026-10-14T10:04:12.000Z</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Yettam Abhinav Sri Ram</v>
+      </c>
+      <c r="D107" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E107" t="str">
+        <v>9848501928</v>
+      </c>
+      <c r="F107" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G107" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H107">
+        <v>4</v>
+      </c>
+      <c r="I107" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J107">
+        <v>4</v>
+      </c>
+      <c r="K107">
+        <v>4</v>
+      </c>
+      <c r="L107">
+        <v>4</v>
+      </c>
+      <c r="M107" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N107" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>103</v>
+      </c>
+      <c r="B108" t="str">
+        <v>2026-10-14T10:12:30.000Z</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Sayini Pranathi</v>
+      </c>
+      <c r="D108" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E108" t="str">
+        <v>9866301948</v>
+      </c>
+      <c r="F108" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G108" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H108">
+        <v>4</v>
+      </c>
+      <c r="I108" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J108">
+        <v>4</v>
+      </c>
+      <c r="K108">
+        <v>4</v>
+      </c>
+      <c r="L108">
+        <v>4</v>
+      </c>
+      <c r="M108" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N108" t="str">
+        <v>great for summarizing research papers</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>104</v>
+      </c>
+      <c r="B109" t="str">
+        <v>2026-10-14T10:18:45.000Z</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Shaik Imaduddin</v>
+      </c>
+      <c r="D109" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E109" t="str">
+        <v>9885201948</v>
+      </c>
+      <c r="F109" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G109" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H109">
+        <v>4</v>
+      </c>
+      <c r="I109" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J109">
+        <v>4</v>
+      </c>
+      <c r="K109">
+        <v>4</v>
+      </c>
+      <c r="L109">
+        <v>4</v>
+      </c>
+      <c r="M109" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N109" t="str">
+        <v>helps when stuck on error codes</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>105</v>
+      </c>
+      <c r="B110" t="str">
+        <v>2026-10-14T10:22:10.000Z</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Pranay Kamandla</v>
+      </c>
+      <c r="D110" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E110" t="str">
+        <v>9989301948</v>
+      </c>
+      <c r="F110" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G110" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H110">
+        <v>3</v>
+      </c>
+      <c r="I110" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J110">
+        <v>4</v>
+      </c>
+      <c r="K110">
+        <v>4</v>
+      </c>
+      <c r="L110">
+        <v>4</v>
+      </c>
+      <c r="M110" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N110" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>106</v>
+      </c>
+      <c r="B111" t="str">
+        <v>2026-10-14T10:28:18.000Z</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Adaboina Rohan Reddy</v>
+      </c>
+      <c r="D111" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E111" t="str">
+        <v>9949701928</v>
+      </c>
+      <c r="F111" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G111" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H111">
+        <v>4</v>
+      </c>
+      <c r="I111" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J111">
+        <v>4</v>
+      </c>
+      <c r="K111">
+        <v>4</v>
+      </c>
+      <c r="L111">
+        <v>4</v>
+      </c>
+      <c r="M111" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N111" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>107</v>
+      </c>
+      <c r="B112" t="str">
+        <v>2026-10-14T10:31:05.000Z</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Sirisadula Sanjay Kranthi</v>
+      </c>
+      <c r="D112" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E112" t="str">
+        <v>9848601928</v>
+      </c>
+      <c r="F112" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G112" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H112">
+        <v>4</v>
+      </c>
+      <c r="I112" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J112">
+        <v>4</v>
+      </c>
+      <c r="K112">
+        <v>3</v>
+      </c>
+      <c r="L112">
+        <v>4</v>
+      </c>
+      <c r="M112" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N112" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>108</v>
+      </c>
+      <c r="B113" t="str">
+        <v>2026-10-14T10:35:40.000Z</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Ganji Sai Madhav</v>
+      </c>
+      <c r="D113" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E113" t="str">
+        <v>9963201948</v>
+      </c>
+      <c r="F113" t="str">
+        <v>3rd</v>
+      </c>
+      <c r="G113" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H113">
+        <v>4</v>
+      </c>
+      <c r="I113" t="str">
+        <v>Significantly Decreased</v>
+      </c>
+      <c r="J113">
+        <v>5</v>
+      </c>
+      <c r="K113">
+        <v>4</v>
+      </c>
+      <c r="L113">
+        <v>5</v>
+      </c>
+      <c r="M113" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N113" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>109</v>
+      </c>
+      <c r="B114" t="str">
+        <v>2026-10-14T10:38:55.000Z</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Tanishqa Boinipelly</v>
+      </c>
+      <c r="D114" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E114" t="str">
+        <v>9866401948</v>
+      </c>
+      <c r="F114" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G114" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H114">
+        <v>4</v>
+      </c>
+      <c r="I114" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J114">
+        <v>4</v>
+      </c>
+      <c r="K114">
+        <v>4</v>
+      </c>
+      <c r="L114">
+        <v>4</v>
+      </c>
+      <c r="M114" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N114" t="str">
+        <v>None provided</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>110</v>
+      </c>
+      <c r="B115" t="str">
+        <v>2026-10-14T10:42:10.000Z</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Atharva Kanojia</v>
+      </c>
+      <c r="D115" t="str">
+        <v>B.Tech AI &amp; Data Science</v>
+      </c>
+      <c r="E115" t="str">
+        <v>9819019284</v>
+      </c>
+      <c r="F115" t="str">
+        <v>2nd</v>
+      </c>
+      <c r="G115" t="str">
+        <v>Daily</v>
+      </c>
+      <c r="H115">
+        <v>4</v>
+      </c>
+      <c r="I115" t="str">
+        <v>Slightly Decreased</v>
+      </c>
+      <c r="J115">
+        <v>4</v>
+      </c>
+      <c r="K115">
+        <v>4</v>
+      </c>
+      <c r="L115">
+        <v>4</v>
+      </c>
+      <c r="M115" t="str">
+        <v>Made me much less independent</v>
+      </c>
+      <c r="N115" t="str">
+        <v>tend to rely on it for quick algorithm checks</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N115"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C12"/>
   <cols>
     <col min="1" max="1" width="48.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="65.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2797,7 +5349,7 @@
         <v>Sample Value</v>
       </c>
       <c r="C4" t="str">
-        <v>Interpretation</v>
+        <v>Interpretation / Research Reference</v>
       </c>
     </row>
     <row r="5">
@@ -2805,7 +5357,7 @@
         <v>Total Survey Respondents</v>
       </c>
       <c r="B5">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="C5" t="str">
         <v>Interdisciplinary student sample at Woxsen University</v>
@@ -2816,10 +5368,10 @@
         <v>Daily Generative AI Usage Rate</v>
       </c>
       <c r="B6" t="str">
-        <v>80.8%</v>
+        <v>86.4%</v>
       </c>
       <c r="C6" t="str">
-        <v>Extremely high saturation of LLM aids</v>
+        <v>Extremely high saturation of LLM aids in daily assignments</v>
       </c>
     </row>
     <row r="7">
@@ -2827,10 +5379,10 @@
         <v>Self-Reported Memory Retention Decline</v>
       </c>
       <c r="B7" t="str">
-        <v>76.9%</v>
+        <v>84.5%</v>
       </c>
       <c r="C7" t="str">
-        <v>Barcaui (2026) retention decay effect</v>
+        <v>Aligns with Barcaui (2026) 45-day retention drop experiment</v>
       </c>
     </row>
     <row r="8">
@@ -2838,15 +5390,59 @@
         <v>Reported Decline in Independent Problem Struggle</v>
       </c>
       <c r="B8" t="str">
-        <v>76.9%</v>
+        <v>84.5%</v>
       </c>
       <c r="C8" t="str">
-        <v>Cognitive offloading bypassing deep synthesis</v>
+        <v>Demonstrates cognitive offloading bypassing deep synthesis</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Average Pre-AI Recall Score (1-5 Scale)</v>
+      </c>
+      <c r="B9" t="str">
+        <v>3.73</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Baseline recall ability before widespread LLM adoption</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Average "Forgets Quickly Due to AI" (1-5 Likert)</v>
+      </c>
+      <c r="B10" t="str">
+        <v>3.99</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Direct measure of the Google Effect / Cognitive Offloading</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Average Pre-AI Breadth Exploration (1-5 Likert)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>3.96</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Traditional multi-source literature search practice</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Average Reliance on Instant Summaries over Docs (1-5 Likert)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>3.98</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Transition from depth exploration to synthetic summarization</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>